<commit_message>
added good / total auto creation
</commit_message>
<xml_diff>
--- a/examples/sample_slos.xlsx
+++ b/examples/sample_slos.xlsx
@@ -362,26 +362,14 @@
 Includes HTTP method and endpoint. Must agree with programs and columns A/B.</t>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
-      <text>
-        <t>spec.objectives[].countMetrics.good.splunkObservability.program
-Complete SignalFlow program for good counts.</t>
-      </text>
-    </comment>
-    <comment ref="AF1" authorId="0" shapeId="0">
-      <text>
-        <t>spec.objectives[].countMetrics.total.splunkObservability.program
-Complete SignalFlow program for total counts.</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SLOCreationTemplate" displayName="SLOCreationTemplate" ref="A1:AF5" headerRowCount="1">
-  <autoFilter ref="A1:AF5"/>
-  <tableColumns count="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SLOCreationTemplate" displayName="SLOCreationTemplate" ref="A1:AD5" headerRowCount="1">
+  <autoFilter ref="A1:AD5"/>
+  <tableColumns count="30">
     <tableColumn id="1" name="endpoint"/>
     <tableColumn id="2" name="http_method"/>
     <tableColumn id="3" name="slo_name"/>
@@ -412,8 +400,6 @@
     <tableColumn id="28" name="splunk_environment"/>
     <tableColumn id="29" name="splunk_service"/>
     <tableColumn id="30" name="splunk_operation"/>
-    <tableColumn id="31" name="good_program"/>
-    <tableColumn id="32" name="total_program"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -708,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF5"/>
+  <dimension ref="A1:AD5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -740,10 +726,7 @@
     <col width="26" customWidth="1" min="27" max="27"/>
     <col width="26" customWidth="1" min="28" max="28"/>
     <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="36" customWidth="1" min="30" max="30"/>
-    <col width="60" customWidth="1" min="31" max="31"/>
-    <col width="60" customWidth="1" min="32" max="32"/>
-    <col width="60" customWidth="1" min="33" max="33"/>
+    <col width="44" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="50" customHeight="1">
@@ -897,16 +880,6 @@
           <t>splunk_operation</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="inlineStr">
-        <is>
-          <t>good_program</t>
-        </is>
-      </c>
-      <c r="AF1" s="6" t="inlineStr">
-        <is>
-          <t>total_program</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="145" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -1047,8 +1020,6 @@
           <t>GET /v1/catalog/items</t>
         </is>
       </c>
-      <c r="AE2" s="7" t="n"/>
-      <c r="AF2" s="7" t="n"/>
     </row>
     <row r="3" ht="145" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
@@ -1189,8 +1160,6 @@
           <t>POST /v1/cart</t>
         </is>
       </c>
-      <c r="AE3" s="7" t="n"/>
-      <c r="AF3" s="7" t="n"/>
     </row>
     <row r="4" ht="145" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -1329,18 +1298,6 @@
           <t>GET /v1/catalog/items</t>
         </is>
       </c>
-      <c r="AE4" s="7" t="inlineStr">
-        <is>
-          <t>good_filter = filter('sf_environment', 'demo-prod') and filter('sf_service', 'demo-store-api') and filter('sf_operation', 'GET /v1/catalog/items') and filter('sf_kind', 'SERVER', 'CONSUMER') and filter('sf_error', 'false') and (not filter('sf_dimensionalized', '*')) and (not filter('sf_serviceMesh', '*'))
-data('spans.count', filter=good_filter).sum().publish(label='good')</t>
-        </is>
-      </c>
-      <c r="AF4" s="7" t="inlineStr">
-        <is>
-          <t>total_filter = filter('sf_environment', 'demo-prod') and filter('sf_service', 'demo-store-api') and filter('sf_operation', 'GET /v1/catalog/items') and filter('sf_kind', 'SERVER', 'CONSUMER') and (not filter('sf_dimensionalized', '*')) and (not filter('sf_serviceMesh', '*'))
-data('spans.count', filter=total_filter).sum().publish(label='total')</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="145" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -1477,18 +1434,6 @@
       <c r="AD5" s="7" t="inlineStr">
         <is>
           <t>POST /v1/cart</t>
-        </is>
-      </c>
-      <c r="AE5" s="7" t="inlineStr">
-        <is>
-          <t>good_filter = filter('sf_environment', 'demo-prod') and filter('sf_service', 'demo-store-api') and filter('sf_operation', 'POST /v1/cart') and filter('sf_kind', 'SERVER', 'CONSUMER') and filter('sf_error', 'false') and (not filter('sf_dimensionalized', '*')) and (not filter('sf_serviceMesh', '*'))
-data('spans.count', filter=good_filter).sum().publish(label='good')</t>
-        </is>
-      </c>
-      <c r="AF5" s="7" t="inlineStr">
-        <is>
-          <t>total_filter = filter('sf_environment', 'demo-prod') and filter('sf_service', 'demo-store-api') and filter('sf_operation', 'POST /v1/cart') and filter('sf_kind', 'SERVER', 'CONSUMER') and (not filter('sf_dimensionalized', '*')) and (not filter('sf_serviceMesh', '*'))
-data('spans.count', filter=total_filter).sum().publish(label='total')</t>
         </is>
       </c>
     </row>
@@ -1588,12 +1533,12 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Raw programs</t>
+          <t>Latency programs</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Python generates latency SignalFlow programs from endpoint, HTTP method, environment, Splunk service and operation. No raw_program input or reference column is needed.</t>
+          <t>Python generates p95 latency SignalFlow from endpoint, method, environment, Splunk service and operation. No program input columns are required.</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1550,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Advanced users may add an optional raw_program column for comparison. It is not required and is not included in this sample.</t>
+          <t>Advanced users can add raw_program, good_program and total_program as optional comparison references. Generated programs are used for output; references are never copied.</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1562,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>good_program and total_program are read directly; environment/service/operation filters must match context columns.</t>
+          <t>Python generates good and total spans.count programs from the context inputs. Good includes sf_error=false; total omits the error filter. Both share span-kind filters and exclusions. incremental is required; sample value is FALSE.</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2227,40 +2172,8 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="90" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>good_program</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>spec.objectives[].countMetrics.good.splunkObservability.program</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Complete SignalFlow program for good counts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>total_program</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>spec.objectives[].countMetrics.total.splunkObservability.program</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Complete SignalFlow program for total counts.</t>
-        </is>
-      </c>
-    </row>
+    <row r="32" ht="90" customHeight="1"/>
+    <row r="33" ht="90" customHeight="1"/>
     <row r="34" ht="62" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>